<commit_message>
Erro no dado indigena denotificaões de violências interpessoais e autoprovocadas e no CS_ESCOL_N no taxa de estupros  e viol domestica
</commit_message>
<xml_diff>
--- a/dados_filtrados/SINAN/notificacoes_viols_agressao_autoprovocadas.xlsx
+++ b/dados_filtrados/SINAN/notificacoes_viols_agressao_autoprovocadas.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="w0Cx07cMcw4kAqa4vtfTTesdatU0JbENSDTMvi1Rs/k="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="cNPtMxJmltjgJ4IDDm07rbZcCBDAMkMsFjFz1nZ7Dog="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Sinan Ano</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t>Amarela</t>
+  </si>
+  <si>
+    <t>Parda</t>
   </si>
   <si>
     <t>Indígena</t>
@@ -170,8 +173,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Tabela_1" name="Tabela_1" id="1">
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K13" displayName="Tabela_1" name="Tabela_1" id="1">
+  <tableColumns count="11">
     <tableColumn name="Sinan Ano" id="1"/>
     <tableColumn name="Agressao" id="2"/>
     <tableColumn name="Autoprovocada" id="3"/>
@@ -181,7 +184,8 @@
     <tableColumn name="Branca" id="7"/>
     <tableColumn name="Preta" id="8"/>
     <tableColumn name="Amarela" id="9"/>
-    <tableColumn name="Indígena" id="10"/>
+    <tableColumn name="Parda" id="10"/>
+    <tableColumn name="Indígena" id="11"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -397,8 +401,9 @@
     <col customWidth="1" min="7" max="7" width="12.86"/>
     <col customWidth="1" min="8" max="8" width="11.29"/>
     <col customWidth="1" min="9" max="9" width="14.14"/>
-    <col customWidth="1" min="10" max="10" width="14.43"/>
-    <col customWidth="1" min="11" max="26" width="8.71"/>
+    <col customWidth="1" min="10" max="10" width="11.86"/>
+    <col customWidth="1" min="11" max="11" width="14.43"/>
+    <col customWidth="1" min="12" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -432,6 +437,9 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="2">
@@ -464,6 +472,9 @@
       <c r="J2" s="2">
         <v>600.0</v>
       </c>
+      <c r="K2" s="2">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="2">
@@ -496,6 +507,9 @@
       <c r="J3" s="2">
         <v>439.0</v>
       </c>
+      <c r="K3" s="2">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="2">
@@ -528,6 +542,9 @@
       <c r="J4" s="2">
         <v>703.0</v>
       </c>
+      <c r="K4" s="2">
+        <v>15.0</v>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="2">
@@ -560,6 +577,9 @@
       <c r="J5" s="2">
         <v>1197.0</v>
       </c>
+      <c r="K5" s="2">
+        <v>21.0</v>
+      </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="2">
@@ -592,6 +612,9 @@
       <c r="J6" s="2">
         <v>1614.0</v>
       </c>
+      <c r="K6" s="2">
+        <v>33.0</v>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="2">
@@ -624,6 +647,9 @@
       <c r="J7" s="2">
         <v>2073.0</v>
       </c>
+      <c r="K7" s="2">
+        <v>24.0</v>
+      </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="2">
@@ -656,6 +682,9 @@
       <c r="J8" s="2">
         <v>2159.0</v>
       </c>
+      <c r="K8" s="2">
+        <v>14.0</v>
+      </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="2">
@@ -688,6 +717,9 @@
       <c r="J9" s="2">
         <v>2635.0</v>
       </c>
+      <c r="K9" s="2">
+        <v>18.0</v>
+      </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="2">
@@ -720,6 +752,9 @@
       <c r="J10" s="2">
         <v>3951.0</v>
       </c>
+      <c r="K10" s="2">
+        <v>28.0</v>
+      </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="2">
@@ -752,6 +787,9 @@
       <c r="J11" s="2">
         <v>6607.0</v>
       </c>
+      <c r="K11" s="2">
+        <v>29.0</v>
+      </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="2">
@@ -784,6 +822,9 @@
       <c r="J12" s="2">
         <v>7626.0</v>
       </c>
+      <c r="K12" s="2">
+        <v>44.0</v>
+      </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="2">
@@ -814,6 +855,9 @@
         <v>0.0</v>
       </c>
       <c r="J13" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="K13" s="2">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>